<commit_message>
Update Excel transaction files with new data for transactions 5 and 6
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 5.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5D150F8-59D7-4B1C-B701-8FD963B52A03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D310A3-C7CA-4D40-86A7-F9BBF452085B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -387,9 +387,6 @@
     <t>26-4-2026</t>
   </si>
   <si>
-    <t>المصريه  لتشكيل المعادن</t>
-  </si>
-  <si>
     <t>العصريه</t>
   </si>
   <si>
@@ -1186,6 +1183,9 @@
   </si>
   <si>
     <t xml:space="preserve">العصريه </t>
+  </si>
+  <si>
+    <t>المصريه لتشكيل المعادن</t>
   </si>
 </sst>
 </file>
@@ -1289,9 +1289,10 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1511,14 +1512,8 @@
     <xf numFmtId="14" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="12" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="2" fontId="9" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1529,10 +1524,16 @@
     <xf numFmtId="2" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1853,7 +1854,7 @@
     </row>
     <row r="3" spans="1:13" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1870,7 +1871,7 @@
     </row>
     <row r="4" spans="1:13" s="23" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A4" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -3573,7 +3574,7 @@
         <v>149122.79999999999</v>
       </c>
       <c r="G49" s="36">
-        <v>1451290</v>
+        <v>1273061</v>
       </c>
       <c r="H49" s="28">
         <v>59830</v>
@@ -3583,7 +3584,7 @@
       </c>
       <c r="J49" s="29"/>
       <c r="K49" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L49" s="27">
         <v>6323</v>
@@ -3605,9 +3606,9 @@
       <c r="D50" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E50" s="37"/>
+      <c r="E50" s="38"/>
       <c r="F50" s="40"/>
-      <c r="G50" s="37"/>
+      <c r="G50" s="38"/>
       <c r="H50" s="28">
         <v>59830</v>
       </c>
@@ -3616,7 +3617,7 @@
       </c>
       <c r="J50" s="29"/>
       <c r="K50" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L50" s="27">
         <v>6323</v>
@@ -3638,9 +3639,9 @@
       <c r="D51" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E51" s="37"/>
+      <c r="E51" s="38"/>
       <c r="F51" s="40"/>
-      <c r="G51" s="37"/>
+      <c r="G51" s="38"/>
       <c r="H51" s="28">
         <v>59830</v>
       </c>
@@ -3649,7 +3650,7 @@
       </c>
       <c r="J51" s="29"/>
       <c r="K51" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L51" s="27">
         <v>6323</v>
@@ -3671,9 +3672,9 @@
       <c r="D52" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E52" s="37"/>
+      <c r="E52" s="38"/>
       <c r="F52" s="40"/>
-      <c r="G52" s="37"/>
+      <c r="G52" s="38"/>
       <c r="H52" s="28">
         <v>59830</v>
       </c>
@@ -3682,7 +3683,7 @@
       </c>
       <c r="J52" s="29"/>
       <c r="K52" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L52" s="27">
         <v>6323</v>
@@ -3704,9 +3705,9 @@
       <c r="D53" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E53" s="37"/>
+      <c r="E53" s="38"/>
       <c r="F53" s="40"/>
-      <c r="G53" s="37"/>
+      <c r="G53" s="38"/>
       <c r="H53" s="28">
         <v>59830</v>
       </c>
@@ -3715,7 +3716,7 @@
       </c>
       <c r="J53" s="29"/>
       <c r="K53" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L53" s="27">
         <v>6323</v>
@@ -3737,9 +3738,9 @@
       <c r="D54" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="E54" s="38"/>
+      <c r="E54" s="37"/>
       <c r="F54" s="41"/>
-      <c r="G54" s="38"/>
+      <c r="G54" s="37"/>
       <c r="H54" s="28">
         <v>59830</v>
       </c>
@@ -3748,7 +3749,7 @@
       </c>
       <c r="J54" s="29"/>
       <c r="K54" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L54" s="27">
         <v>6323</v>
@@ -3762,7 +3763,7 @@
         <v>51</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>115</v>
@@ -3787,7 +3788,7 @@
       </c>
       <c r="J55" s="8"/>
       <c r="K55" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L55" s="4">
         <v>6324</v>
@@ -3801,7 +3802,7 @@
         <v>52</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>116</v>
@@ -3826,7 +3827,7 @@
       </c>
       <c r="J56" s="8"/>
       <c r="K56" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L56" s="4">
         <v>6324</v>
@@ -3840,7 +3841,7 @@
         <v>53</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>117</v>
@@ -3865,7 +3866,7 @@
       </c>
       <c r="J57" s="8"/>
       <c r="K57" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="L57" s="4">
         <v>6324</v>
@@ -3904,7 +3905,7 @@
       </c>
       <c r="J58" s="29"/>
       <c r="K58" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L58" s="27">
         <v>6325</v>
@@ -3930,7 +3931,7 @@
         <v>95</v>
       </c>
       <c r="F59" s="40"/>
-      <c r="G59" s="37"/>
+      <c r="G59" s="38"/>
       <c r="H59" s="27">
         <v>59837</v>
       </c>
@@ -3939,7 +3940,7 @@
       </c>
       <c r="J59" s="29"/>
       <c r="K59" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L59" s="27">
         <v>6325</v>
@@ -3953,10 +3954,10 @@
         <v>56</v>
       </c>
       <c r="B60" s="26" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C60" s="27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D60" s="27" t="s">
         <v>16</v>
@@ -3965,7 +3966,7 @@
         <v>88</v>
       </c>
       <c r="F60" s="40"/>
-      <c r="G60" s="37"/>
+      <c r="G60" s="38"/>
       <c r="H60" s="27">
         <v>59837</v>
       </c>
@@ -3974,7 +3975,7 @@
       </c>
       <c r="J60" s="29"/>
       <c r="K60" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L60" s="27">
         <v>6325</v>
@@ -3988,10 +3989,10 @@
         <v>57</v>
       </c>
       <c r="B61" s="26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C61" s="27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D61" s="27" t="s">
         <v>16</v>
@@ -4000,7 +4001,7 @@
         <v>80</v>
       </c>
       <c r="F61" s="41"/>
-      <c r="G61" s="38"/>
+      <c r="G61" s="37"/>
       <c r="H61" s="27">
         <v>59837</v>
       </c>
@@ -4009,7 +4010,7 @@
       </c>
       <c r="J61" s="29"/>
       <c r="K61" s="27" t="s">
-        <v>119</v>
+        <v>385</v>
       </c>
       <c r="L61" s="27">
         <v>6325</v>
@@ -4023,10 +4024,10 @@
         <v>58</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D62" s="4" t="s">
         <v>16</v>
@@ -4048,7 +4049,7 @@
       </c>
       <c r="J62" s="8"/>
       <c r="K62" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L62" s="4">
         <v>6326</v>
@@ -4062,10 +4063,10 @@
         <v>59</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D63" s="4" t="s">
         <v>16</v>
@@ -4087,7 +4088,7 @@
       </c>
       <c r="J63" s="8"/>
       <c r="K63" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L63" s="4">
         <v>6326</v>
@@ -4101,10 +4102,10 @@
         <v>60</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D64" s="4" t="s">
         <v>16</v>
@@ -4126,7 +4127,7 @@
       </c>
       <c r="J64" s="8"/>
       <c r="K64" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L64" s="4">
         <v>6327</v>
@@ -4140,10 +4141,10 @@
         <v>61</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D65" s="4" t="s">
         <v>16</v>
@@ -4165,7 +4166,7 @@
       </c>
       <c r="J65" s="8"/>
       <c r="K65" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L65" s="4">
         <v>6327</v>
@@ -4179,13 +4180,13 @@
         <v>62</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C66" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D66" s="4" t="s">
         <v>136</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>137</v>
       </c>
       <c r="E66" s="4">
         <v>50</v>
@@ -4204,7 +4205,7 @@
       </c>
       <c r="J66" s="8"/>
       <c r="K66" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L66" s="4">
         <v>6327</v>
@@ -4218,10 +4219,10 @@
         <v>63</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>16</v>
@@ -4243,7 +4244,7 @@
       </c>
       <c r="J67" s="8"/>
       <c r="K67" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L67" s="4">
         <v>6327</v>
@@ -4257,10 +4258,10 @@
         <v>64</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>16</v>
@@ -4282,7 +4283,7 @@
       </c>
       <c r="J68" s="8"/>
       <c r="K68" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L68" s="4">
         <v>6327</v>
@@ -4296,10 +4297,10 @@
         <v>65</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D69" s="4" t="s">
         <v>16</v>
@@ -4321,7 +4322,7 @@
       </c>
       <c r="J69" s="8"/>
       <c r="K69" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L69" s="4">
         <v>6327</v>
@@ -4335,10 +4336,10 @@
         <v>66</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D70" s="4" t="s">
         <v>16</v>
@@ -4360,7 +4361,7 @@
       </c>
       <c r="J70" s="8"/>
       <c r="K70" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L70" s="4">
         <v>6327</v>
@@ -4374,10 +4375,10 @@
         <v>67</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D71" s="4" t="s">
         <v>16</v>
@@ -4399,7 +4400,7 @@
       </c>
       <c r="J71" s="8"/>
       <c r="K71" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L71" s="4">
         <v>6327</v>
@@ -4413,10 +4414,10 @@
         <v>69</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D72" s="4" t="s">
         <v>16</v>
@@ -4438,7 +4439,7 @@
       </c>
       <c r="J72" s="8"/>
       <c r="K72" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L72" s="4">
         <v>6327</v>
@@ -4452,10 +4453,10 @@
         <v>70</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D73" s="4" t="s">
         <v>16</v>
@@ -4477,7 +4478,7 @@
       </c>
       <c r="J73" s="8"/>
       <c r="K73" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L73" s="4">
         <v>6328</v>
@@ -4491,10 +4492,10 @@
         <v>71</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D74" s="4" t="s">
         <v>16</v>
@@ -4516,7 +4517,7 @@
       </c>
       <c r="J74" s="8"/>
       <c r="K74" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L74" s="4">
         <v>6328</v>
@@ -4530,10 +4531,10 @@
         <v>72</v>
       </c>
       <c r="B75" s="12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>16</v>
@@ -4555,7 +4556,7 @@
       </c>
       <c r="J75" s="8"/>
       <c r="K75" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L75" s="4">
         <v>6328</v>
@@ -4569,10 +4570,10 @@
         <v>73</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D76" s="4" t="s">
         <v>16</v>
@@ -4594,7 +4595,7 @@
       </c>
       <c r="J76" s="8"/>
       <c r="K76" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L76" s="4">
         <v>6328</v>
@@ -4608,13 +4609,13 @@
         <v>74</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C77" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="D77" s="4" t="s">
         <v>161</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>162</v>
       </c>
       <c r="E77" s="4">
         <v>45.5</v>
@@ -4633,7 +4634,7 @@
       </c>
       <c r="J77" s="8"/>
       <c r="K77" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L77" s="4">
         <v>6329</v>
@@ -4647,10 +4648,10 @@
         <v>75</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>16</v>
@@ -4672,7 +4673,7 @@
       </c>
       <c r="J78" s="8"/>
       <c r="K78" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L78" s="4">
         <v>6330</v>
@@ -4686,10 +4687,10 @@
         <v>76</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>16</v>
@@ -4707,11 +4708,11 @@
         <v>6525</v>
       </c>
       <c r="I79" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J79" s="8"/>
       <c r="K79" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L79" s="4">
         <v>6331</v>
@@ -4725,10 +4726,10 @@
         <v>77</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D80" s="4" t="s">
         <v>16</v>
@@ -4746,11 +4747,11 @@
         <v>6525</v>
       </c>
       <c r="I80" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J80" s="8"/>
       <c r="K80" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L80" s="4">
         <v>6331</v>
@@ -4764,10 +4765,10 @@
         <v>78</v>
       </c>
       <c r="B81" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D81" s="4" t="s">
         <v>16</v>
@@ -4785,11 +4786,11 @@
         <v>6526</v>
       </c>
       <c r="I81" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J81" s="8"/>
       <c r="K81" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L81" s="4">
         <v>6332</v>
@@ -4803,10 +4804,10 @@
         <v>79</v>
       </c>
       <c r="B82" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D82" s="4" t="s">
         <v>16</v>
@@ -4824,11 +4825,11 @@
         <v>6526</v>
       </c>
       <c r="I82" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J82" s="8"/>
       <c r="K82" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L82" s="4">
         <v>6332</v>
@@ -4842,10 +4843,10 @@
         <v>80</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D83" s="4" t="s">
         <v>16</v>
@@ -4863,11 +4864,11 @@
         <v>6526</v>
       </c>
       <c r="I83" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J83" s="8"/>
       <c r="K83" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L83" s="4">
         <v>6332</v>
@@ -4881,10 +4882,10 @@
         <v>81</v>
       </c>
       <c r="B84" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C84" s="15" t="s">
         <v>203</v>
-      </c>
-      <c r="C84" s="15" t="s">
-        <v>204</v>
       </c>
       <c r="D84" s="4" t="s">
         <v>16</v>
@@ -4902,11 +4903,11 @@
         <v>929</v>
       </c>
       <c r="I84" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J84" s="8"/>
       <c r="K84" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L84" s="4">
         <v>6333</v>
@@ -4920,10 +4921,10 @@
         <v>82</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D85" s="4" t="s">
         <v>16</v>
@@ -4941,11 +4942,11 @@
         <v>929</v>
       </c>
       <c r="I85" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J85" s="8"/>
       <c r="K85" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L85" s="4">
         <v>6333</v>
@@ -4959,10 +4960,10 @@
         <v>83</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D86" s="4" t="s">
         <v>16</v>
@@ -4980,11 +4981,11 @@
         <v>929</v>
       </c>
       <c r="I86" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J86" s="8"/>
       <c r="K86" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L86" s="4">
         <v>6333</v>
@@ -4998,10 +4999,10 @@
         <v>84</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D87" s="4" t="s">
         <v>16</v>
@@ -5019,11 +5020,11 @@
         <v>929</v>
       </c>
       <c r="I87" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J87" s="8"/>
       <c r="K87" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L87" s="4">
         <v>6333</v>
@@ -5037,7 +5038,7 @@
         <v>85</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>115</v>
@@ -5058,11 +5059,11 @@
         <v>929</v>
       </c>
       <c r="I88" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J88" s="8"/>
       <c r="K88" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L88" s="4">
         <v>6333</v>
@@ -5076,10 +5077,10 @@
         <v>86</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D89" s="4" t="s">
         <v>16</v>
@@ -5097,11 +5098,11 @@
         <v>929</v>
       </c>
       <c r="I89" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J89" s="8"/>
       <c r="K89" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L89" s="4">
         <v>6333</v>
@@ -5115,7 +5116,7 @@
         <v>87</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>116</v>
@@ -5136,11 +5137,11 @@
         <v>929</v>
       </c>
       <c r="I90" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J90" s="8"/>
       <c r="K90" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L90" s="4">
         <v>6333</v>
@@ -5154,10 +5155,10 @@
         <v>88</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D91" s="4" t="s">
         <v>16</v>
@@ -5175,11 +5176,11 @@
         <v>929</v>
       </c>
       <c r="I91" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J91" s="8"/>
       <c r="K91" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L91" s="4">
         <v>6333</v>
@@ -5193,10 +5194,10 @@
         <v>89</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D92" s="4" t="s">
         <v>16</v>
@@ -5214,11 +5215,11 @@
         <v>929</v>
       </c>
       <c r="I92" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J92" s="8"/>
       <c r="K92" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L92" s="4">
         <v>6333</v>
@@ -5232,10 +5233,10 @@
         <v>90</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D93" s="4" t="s">
         <v>16</v>
@@ -5253,11 +5254,11 @@
         <v>929</v>
       </c>
       <c r="I93" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J93" s="8"/>
       <c r="K93" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L93" s="4">
         <v>6333</v>
@@ -5271,10 +5272,10 @@
         <v>91</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D94" s="4" t="s">
         <v>16</v>
@@ -5292,11 +5293,11 @@
         <v>929</v>
       </c>
       <c r="I94" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J94" s="8"/>
       <c r="K94" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L94" s="4">
         <v>6333</v>
@@ -5310,10 +5311,10 @@
         <v>92</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D95" s="4" t="s">
         <v>16</v>
@@ -5331,11 +5332,11 @@
         <v>929</v>
       </c>
       <c r="I95" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J95" s="8"/>
       <c r="K95" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L95" s="4">
         <v>6333</v>
@@ -5349,10 +5350,10 @@
         <v>93</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D96" s="4" t="s">
         <v>16</v>
@@ -5370,11 +5371,11 @@
         <v>929</v>
       </c>
       <c r="I96" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J96" s="8"/>
       <c r="K96" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L96" s="4">
         <v>6333</v>
@@ -5388,10 +5389,10 @@
         <v>94</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D97" s="4" t="s">
         <v>16</v>
@@ -5409,11 +5410,11 @@
         <v>929</v>
       </c>
       <c r="I97" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J97" s="8"/>
       <c r="K97" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L97" s="4">
         <v>6333</v>
@@ -5427,10 +5428,10 @@
         <v>95</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D98" s="4" t="s">
         <v>16</v>
@@ -5448,11 +5449,11 @@
         <v>928</v>
       </c>
       <c r="I98" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J98" s="8"/>
       <c r="K98" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L98" s="4">
         <v>6335</v>
@@ -5466,10 +5467,10 @@
         <v>96</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D99" s="4" t="s">
         <v>16</v>
@@ -5487,11 +5488,11 @@
         <v>928</v>
       </c>
       <c r="I99" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J99" s="8"/>
       <c r="K99" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L99" s="4">
         <v>6335</v>
@@ -5505,13 +5506,13 @@
         <v>97</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E100" s="4">
         <v>6</v>
@@ -5526,11 +5527,11 @@
         <v>928</v>
       </c>
       <c r="I100" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J100" s="8"/>
       <c r="K100" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L100" s="4">
         <v>6335</v>
@@ -5544,10 +5545,10 @@
         <v>98</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D101" s="4" t="s">
         <v>16</v>
@@ -5565,11 +5566,11 @@
         <v>928</v>
       </c>
       <c r="I101" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J101" s="8"/>
       <c r="K101" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L101" s="4">
         <v>6335</v>
@@ -5583,10 +5584,10 @@
         <v>99</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D102" s="4" t="s">
         <v>16</v>
@@ -5604,11 +5605,11 @@
         <v>928</v>
       </c>
       <c r="I102" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J102" s="8"/>
       <c r="K102" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L102" s="4">
         <v>6335</v>
@@ -5622,10 +5623,10 @@
         <v>100</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D103" s="4" t="s">
         <v>16</v>
@@ -5643,11 +5644,11 @@
         <v>928</v>
       </c>
       <c r="I103" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J103" s="8"/>
       <c r="K103" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L103" s="4">
         <v>6335</v>
@@ -5661,10 +5662,10 @@
         <v>101</v>
       </c>
       <c r="B104" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="C104" s="15" t="s">
         <v>203</v>
-      </c>
-      <c r="C104" s="15" t="s">
-        <v>204</v>
       </c>
       <c r="D104" s="4" t="s">
         <v>16</v>
@@ -5682,11 +5683,11 @@
         <v>928</v>
       </c>
       <c r="I104" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J104" s="8"/>
       <c r="K104" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L104" s="4">
         <v>6335</v>
@@ -5700,13 +5701,13 @@
         <v>102</v>
       </c>
       <c r="B105" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E105" s="4">
         <v>50</v>
@@ -5721,11 +5722,11 @@
         <v>928</v>
       </c>
       <c r="I105" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J105" s="8"/>
       <c r="K105" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L105" s="4">
         <v>6335</v>
@@ -5739,10 +5740,10 @@
         <v>103</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D106" s="4" t="s">
         <v>16</v>
@@ -5760,11 +5761,11 @@
         <v>928</v>
       </c>
       <c r="I106" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J106" s="8"/>
       <c r="K106" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L106" s="4">
         <v>6335</v>
@@ -5778,10 +5779,10 @@
         <v>104</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D107" s="4" t="s">
         <v>16</v>
@@ -5799,11 +5800,11 @@
         <v>928</v>
       </c>
       <c r="I107" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J107" s="8"/>
       <c r="K107" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L107" s="4">
         <v>6335</v>
@@ -5817,13 +5818,13 @@
         <v>105</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E108" s="4">
         <v>50</v>
@@ -5838,11 +5839,11 @@
         <v>928</v>
       </c>
       <c r="I108" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J108" s="8"/>
       <c r="K108" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L108" s="4">
         <v>6335</v>
@@ -5856,13 +5857,13 @@
         <v>106</v>
       </c>
       <c r="B109" s="12" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E109" s="4">
         <v>50</v>
@@ -5877,11 +5878,11 @@
         <v>81</v>
       </c>
       <c r="I109" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J109" s="8"/>
       <c r="K109" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L109" s="4">
         <v>6336</v>
@@ -5895,10 +5896,10 @@
         <v>107</v>
       </c>
       <c r="B110" s="12" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D110" s="4" t="s">
         <v>16</v>
@@ -5916,11 +5917,11 @@
         <v>81</v>
       </c>
       <c r="I110" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J110" s="8"/>
       <c r="K110" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L110" s="4">
         <v>6336</v>
@@ -5934,10 +5935,10 @@
         <v>108</v>
       </c>
       <c r="B111" s="12" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D111" s="4" t="s">
         <v>16</v>
@@ -5955,11 +5956,11 @@
         <v>81</v>
       </c>
       <c r="I111" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J111" s="8"/>
       <c r="K111" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L111" s="4">
         <v>6336</v>
@@ -5973,10 +5974,10 @@
         <v>109</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D112" s="4" t="s">
         <v>16</v>
@@ -5994,11 +5995,11 @@
         <v>81</v>
       </c>
       <c r="I112" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J112" s="8"/>
       <c r="K112" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L112" s="4">
         <v>6336</v>
@@ -6012,10 +6013,10 @@
         <v>110</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D113" s="4" t="s">
         <v>16</v>
@@ -6033,11 +6034,11 @@
         <v>81</v>
       </c>
       <c r="I113" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J113" s="8"/>
       <c r="K113" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L113" s="4">
         <v>6336</v>
@@ -6051,10 +6052,10 @@
         <v>111</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D114" s="4" t="s">
         <v>16</v>
@@ -6072,11 +6073,11 @@
         <v>81</v>
       </c>
       <c r="I114" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J114" s="8"/>
       <c r="K114" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L114" s="4">
         <v>6336</v>
@@ -6090,10 +6091,10 @@
         <v>113</v>
       </c>
       <c r="B115" s="12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C115" s="17" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D115" s="17" t="s">
         <v>16</v>
@@ -6111,11 +6112,11 @@
         <v>1755</v>
       </c>
       <c r="I115" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J115" s="19"/>
       <c r="K115" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L115" s="17">
         <v>6337</v>
@@ -6129,10 +6130,10 @@
         <v>114</v>
       </c>
       <c r="B116" s="12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C116" s="17" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D116" s="17" t="s">
         <v>16</v>
@@ -6150,11 +6151,11 @@
         <v>1755</v>
       </c>
       <c r="I116" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J116" s="19"/>
       <c r="K116" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L116" s="17">
         <v>6337</v>
@@ -6168,10 +6169,10 @@
         <v>115</v>
       </c>
       <c r="B117" s="12" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C117" s="17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D117" s="17" t="s">
         <v>16</v>
@@ -6189,11 +6190,11 @@
         <v>1755</v>
       </c>
       <c r="I117" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J117" s="19"/>
       <c r="K117" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L117" s="17">
         <v>6337</v>
@@ -6207,10 +6208,10 @@
         <v>116</v>
       </c>
       <c r="B118" s="12" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C118" s="17" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D118" s="17" t="s">
         <v>16</v>
@@ -6228,11 +6229,11 @@
         <v>1755</v>
       </c>
       <c r="I118" s="18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J118" s="19"/>
       <c r="K118" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L118" s="17">
         <v>6337</v>
@@ -6246,10 +6247,10 @@
         <v>117</v>
       </c>
       <c r="B119" s="12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D119" s="4" t="s">
         <v>16</v>
@@ -6267,11 +6268,11 @@
         <v>85</v>
       </c>
       <c r="I119" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J119" s="8"/>
       <c r="K119" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L119" s="4">
         <v>6339</v>
@@ -6285,10 +6286,10 @@
         <v>118</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D120" s="4" t="s">
         <v>16</v>
@@ -6306,11 +6307,11 @@
         <v>85</v>
       </c>
       <c r="I120" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J120" s="8"/>
       <c r="K120" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L120" s="4">
         <v>6339</v>
@@ -6324,10 +6325,10 @@
         <v>119</v>
       </c>
       <c r="B121" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D121" s="4" t="s">
         <v>16</v>
@@ -6345,11 +6346,11 @@
         <v>85</v>
       </c>
       <c r="I121" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J121" s="8"/>
       <c r="K121" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L121" s="4">
         <v>6339</v>
@@ -6363,10 +6364,10 @@
         <v>120</v>
       </c>
       <c r="B122" s="12" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D122" s="4" t="s">
         <v>16</v>
@@ -6384,11 +6385,11 @@
         <v>85</v>
       </c>
       <c r="I122" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J122" s="8"/>
       <c r="K122" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L122" s="4">
         <v>6339</v>
@@ -6402,10 +6403,10 @@
         <v>121</v>
       </c>
       <c r="B123" s="13" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D123" s="4" t="s">
         <v>16</v>
@@ -6423,11 +6424,11 @@
         <v>85</v>
       </c>
       <c r="I123" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J123" s="8"/>
       <c r="K123" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L123" s="4">
         <v>6339</v>
@@ -6441,10 +6442,10 @@
         <v>122</v>
       </c>
       <c r="B124" s="13" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D124" s="4" t="s">
         <v>16</v>
@@ -6462,11 +6463,11 @@
         <v>85</v>
       </c>
       <c r="I124" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J124" s="8"/>
       <c r="K124" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L124" s="4">
         <v>6339</v>
@@ -6480,10 +6481,10 @@
         <v>123</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D125" s="4" t="s">
         <v>16</v>
@@ -6501,11 +6502,11 @@
         <v>86</v>
       </c>
       <c r="I125" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J125" s="8"/>
       <c r="K125" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L125" s="4">
         <v>6340</v>
@@ -6519,10 +6520,10 @@
         <v>124</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D126" s="4" t="s">
         <v>16</v>
@@ -6540,11 +6541,11 @@
         <v>86</v>
       </c>
       <c r="I126" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J126" s="8"/>
       <c r="K126" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L126" s="4">
         <v>6340</v>
@@ -6558,10 +6559,10 @@
         <v>125</v>
       </c>
       <c r="B127" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D127" s="4" t="s">
         <v>16</v>
@@ -6579,11 +6580,11 @@
         <v>86</v>
       </c>
       <c r="I127" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J127" s="8"/>
       <c r="K127" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L127" s="4">
         <v>6340</v>
@@ -6597,10 +6598,10 @@
         <v>126</v>
       </c>
       <c r="B128" s="12" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C128" s="21" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D128" s="4" t="s">
         <v>16</v>
@@ -6618,11 +6619,11 @@
         <v>86</v>
       </c>
       <c r="I128" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J128" s="8"/>
       <c r="K128" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L128" s="4">
         <v>6340</v>
@@ -6636,10 +6637,10 @@
         <v>127</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D129" s="4" t="s">
         <v>16</v>
@@ -6657,11 +6658,11 @@
         <v>722</v>
       </c>
       <c r="I129" s="9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J129" s="8"/>
       <c r="K129" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="L129" s="4">
         <v>6341</v>
@@ -6675,10 +6676,10 @@
         <v>128</v>
       </c>
       <c r="B130" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D130" s="4" t="s">
         <v>16</v>
@@ -6696,17 +6697,17 @@
         <v>89</v>
       </c>
       <c r="I130" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J130" s="8"/>
       <c r="K130" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L130" s="4">
         <v>6342</v>
       </c>
       <c r="M130" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="131" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6714,10 +6715,10 @@
         <v>129</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D131" s="4" t="s">
         <v>16</v>
@@ -6735,17 +6736,17 @@
         <v>89</v>
       </c>
       <c r="I131" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J131" s="8"/>
       <c r="K131" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L131" s="4">
         <v>6342</v>
       </c>
       <c r="M131" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="132" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6753,10 +6754,10 @@
         <v>130</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D132" s="4" t="s">
         <v>16</v>
@@ -6774,17 +6775,17 @@
         <v>89</v>
       </c>
       <c r="I132" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J132" s="8"/>
       <c r="K132" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L132" s="4">
         <v>6342</v>
       </c>
       <c r="M132" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="133" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6792,10 +6793,10 @@
         <v>131</v>
       </c>
       <c r="B133" s="12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D133" s="16" t="s">
         <v>16</v>
@@ -6813,11 +6814,11 @@
         <v>19241</v>
       </c>
       <c r="I133" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J133" s="8"/>
       <c r="K133" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="L133" s="4">
         <v>6343</v>
@@ -6834,13 +6835,13 @@
         <v>111</v>
       </c>
       <c r="C134" s="27" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D134" s="28" t="s">
-        <v>60</v>
+        <v>161</v>
       </c>
       <c r="E134" s="36">
-        <v>109.649</v>
+        <v>2101</v>
       </c>
       <c r="F134" s="36">
         <v>109.649</v>
@@ -6851,12 +6852,12 @@
       <c r="H134" s="28">
         <v>59846</v>
       </c>
-      <c r="I134" s="35" t="s">
-        <v>168</v>
+      <c r="I134" s="33" t="s">
+        <v>167</v>
       </c>
       <c r="J134" s="29"/>
-      <c r="K134" s="34" t="s">
-        <v>119</v>
+      <c r="K134" s="32" t="s">
+        <v>385</v>
       </c>
       <c r="L134" s="27">
         <v>6338</v>
@@ -6870,26 +6871,26 @@
         <v>133</v>
       </c>
       <c r="B135" s="26" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C135" s="27" t="s">
-        <v>276</v>
-      </c>
-      <c r="D135" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="E135" s="37"/>
-      <c r="F135" s="37"/>
-      <c r="G135" s="37"/>
+        <v>275</v>
+      </c>
+      <c r="D135" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="E135" s="38"/>
+      <c r="F135" s="38"/>
+      <c r="G135" s="38"/>
       <c r="H135" s="28">
         <v>59846</v>
       </c>
-      <c r="I135" s="35" t="s">
-        <v>380</v>
+      <c r="I135" s="33" t="s">
+        <v>379</v>
       </c>
       <c r="J135" s="29"/>
-      <c r="K135" s="34" t="s">
-        <v>119</v>
+      <c r="K135" s="32" t="s">
+        <v>385</v>
       </c>
       <c r="L135" s="27">
         <v>6338</v>
@@ -6908,21 +6909,21 @@
       <c r="C136" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="D136" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="E136" s="37"/>
-      <c r="F136" s="37"/>
-      <c r="G136" s="37"/>
+      <c r="D136" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="E136" s="38"/>
+      <c r="F136" s="38"/>
+      <c r="G136" s="38"/>
       <c r="H136" s="28">
         <v>59846</v>
       </c>
-      <c r="I136" s="35" t="s">
-        <v>381</v>
+      <c r="I136" s="33" t="s">
+        <v>380</v>
       </c>
       <c r="J136" s="29"/>
-      <c r="K136" s="34" t="s">
-        <v>119</v>
+      <c r="K136" s="32" t="s">
+        <v>385</v>
       </c>
       <c r="L136" s="27">
         <v>6338</v>
@@ -6935,27 +6936,27 @@
       <c r="A137" s="25">
         <v>135</v>
       </c>
-      <c r="B137" s="32" t="s">
+      <c r="B137" s="31" t="s">
+        <v>337</v>
+      </c>
+      <c r="C137" s="35" t="s">
         <v>338</v>
       </c>
-      <c r="C137" s="33" t="s">
-        <v>339</v>
-      </c>
-      <c r="D137" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="E137" s="38"/>
-      <c r="F137" s="38"/>
-      <c r="G137" s="38"/>
+      <c r="D137" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="E137" s="37"/>
+      <c r="F137" s="37"/>
+      <c r="G137" s="37"/>
       <c r="H137" s="28">
         <v>59846</v>
       </c>
-      <c r="I137" s="35" t="s">
-        <v>382</v>
+      <c r="I137" s="33" t="s">
+        <v>381</v>
       </c>
       <c r="J137" s="29"/>
-      <c r="K137" s="34" t="s">
-        <v>119</v>
+      <c r="K137" s="32" t="s">
+        <v>385</v>
       </c>
       <c r="L137" s="27">
         <v>6338</v>
@@ -6969,32 +6970,32 @@
         <v>136</v>
       </c>
       <c r="B138" s="26" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C138" s="27" t="s">
-        <v>277</v>
-      </c>
-      <c r="D138" s="31" t="s">
-        <v>60</v>
+        <v>276</v>
+      </c>
+      <c r="D138" s="34" t="s">
+        <v>161</v>
       </c>
       <c r="E138" s="36">
-        <v>2.101</v>
+        <v>13828</v>
       </c>
       <c r="F138" s="36">
         <v>157.89400000000001</v>
       </c>
       <c r="G138" s="36">
-        <v>283368.40000000002</v>
+        <v>2183368.4</v>
       </c>
       <c r="H138" s="28">
         <v>59846</v>
       </c>
-      <c r="I138" s="35" t="s">
-        <v>383</v>
+      <c r="I138" s="33" t="s">
+        <v>382</v>
       </c>
       <c r="J138" s="29"/>
-      <c r="K138" s="34" t="s">
-        <v>119</v>
+      <c r="K138" s="32" t="s">
+        <v>385</v>
       </c>
       <c r="L138" s="27">
         <v>6338</v>
@@ -7011,23 +7012,23 @@
         <v>113</v>
       </c>
       <c r="C139" s="27" t="s">
-        <v>278</v>
-      </c>
-      <c r="D139" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="E139" s="38"/>
-      <c r="F139" s="38"/>
-      <c r="G139" s="38"/>
+        <v>277</v>
+      </c>
+      <c r="D139" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="E139" s="37"/>
+      <c r="F139" s="37"/>
+      <c r="G139" s="37"/>
       <c r="H139" s="28">
         <v>59846</v>
       </c>
-      <c r="I139" s="35" t="s">
-        <v>384</v>
+      <c r="I139" s="33" t="s">
+        <v>383</v>
       </c>
       <c r="J139" s="29"/>
-      <c r="K139" s="34" t="s">
-        <v>119</v>
+      <c r="K139" s="32" t="s">
+        <v>385</v>
       </c>
       <c r="L139" s="27">
         <v>6338</v>
@@ -7041,10 +7042,10 @@
         <v>138</v>
       </c>
       <c r="B140" s="11" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D140" s="4" t="s">
         <v>16</v>
@@ -7066,13 +7067,13 @@
       </c>
       <c r="J140" s="8"/>
       <c r="K140" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="L140" s="4">
         <v>6344</v>
       </c>
       <c r="M140" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="141" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7080,10 +7081,10 @@
         <v>139</v>
       </c>
       <c r="B141" s="24" t="s">
+        <v>341</v>
+      </c>
+      <c r="C141" s="14" t="s">
         <v>342</v>
-      </c>
-      <c r="C141" s="14" t="s">
-        <v>343</v>
       </c>
       <c r="D141" s="4" t="s">
         <v>16</v>
@@ -7105,13 +7106,13 @@
       </c>
       <c r="J141" s="8"/>
       <c r="K141" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L141" s="4">
         <v>6345</v>
       </c>
       <c r="M141" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="142" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7119,10 +7120,10 @@
         <v>140</v>
       </c>
       <c r="B142" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D142" s="4" t="s">
         <v>16</v>
@@ -7144,13 +7145,13 @@
       </c>
       <c r="J142" s="8"/>
       <c r="K142" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L142" s="4">
         <v>6345</v>
       </c>
       <c r="M142" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="143" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7158,10 +7159,10 @@
         <v>141</v>
       </c>
       <c r="B143" s="12" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D143" s="4" t="s">
         <v>16</v>
@@ -7183,13 +7184,13 @@
       </c>
       <c r="J143" s="8"/>
       <c r="K143" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L143" s="4">
         <v>6345</v>
       </c>
       <c r="M143" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="144" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7197,10 +7198,10 @@
         <v>142</v>
       </c>
       <c r="B144" s="12" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D144" s="4" t="s">
         <v>16</v>
@@ -7222,13 +7223,13 @@
       </c>
       <c r="J144" s="8"/>
       <c r="K144" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L144" s="4">
         <v>6345</v>
       </c>
       <c r="M144" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="145" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7236,10 +7237,10 @@
         <v>143</v>
       </c>
       <c r="B145" s="12" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D145" s="4" t="s">
         <v>16</v>
@@ -7261,13 +7262,13 @@
       </c>
       <c r="J145" s="8"/>
       <c r="K145" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L145" s="4">
         <v>6345</v>
       </c>
       <c r="M145" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="146" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7276,7 +7277,7 @@
       </c>
       <c r="B146" s="6"/>
       <c r="C146" s="4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D146" s="4" t="s">
         <v>16</v>
@@ -7298,13 +7299,13 @@
       </c>
       <c r="J146" s="8"/>
       <c r="K146" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L146" s="4">
         <v>6345</v>
       </c>
       <c r="M146" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="147" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7312,10 +7313,10 @@
         <v>145</v>
       </c>
       <c r="B147" s="12" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D147" s="4" t="s">
         <v>16</v>
@@ -7337,13 +7338,13 @@
       </c>
       <c r="J147" s="8"/>
       <c r="K147" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L147" s="4">
         <v>6345</v>
       </c>
       <c r="M147" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="148" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7351,10 +7352,10 @@
         <v>146</v>
       </c>
       <c r="B148" s="12" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D148" s="4" t="s">
         <v>16</v>
@@ -7376,13 +7377,13 @@
       </c>
       <c r="J148" s="8"/>
       <c r="K148" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L148" s="4">
         <v>6345</v>
       </c>
       <c r="M148" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="149" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7390,10 +7391,10 @@
         <v>147</v>
       </c>
       <c r="B149" s="12" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D149" s="4" t="s">
         <v>16</v>
@@ -7415,13 +7416,13 @@
       </c>
       <c r="J149" s="8"/>
       <c r="K149" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L149" s="4">
         <v>6345</v>
       </c>
       <c r="M149" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="150" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7429,10 +7430,10 @@
         <v>148</v>
       </c>
       <c r="B150" s="12" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D150" s="4" t="s">
         <v>16</v>
@@ -7454,13 +7455,13 @@
       </c>
       <c r="J150" s="8"/>
       <c r="K150" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L150" s="4">
         <v>6345</v>
       </c>
       <c r="M150" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="151" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7468,10 +7469,10 @@
         <v>149</v>
       </c>
       <c r="B151" s="11" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D151" s="4" t="s">
         <v>16</v>
@@ -7493,13 +7494,13 @@
       </c>
       <c r="J151" s="8"/>
       <c r="K151" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L151" s="4">
         <v>6347</v>
       </c>
       <c r="M151" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="152" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7507,10 +7508,10 @@
         <v>150</v>
       </c>
       <c r="B152" s="11" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D152" s="4" t="s">
         <v>16</v>
@@ -7532,13 +7533,13 @@
       </c>
       <c r="J152" s="8"/>
       <c r="K152" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L152" s="4">
         <v>6347</v>
       </c>
       <c r="M152" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="153" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7546,10 +7547,10 @@
         <v>151</v>
       </c>
       <c r="B153" s="12" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D153" s="4" t="s">
         <v>16</v>
@@ -7571,13 +7572,13 @@
       </c>
       <c r="J153" s="8"/>
       <c r="K153" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L153" s="4">
         <v>6347</v>
       </c>
       <c r="M153" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="154" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7585,10 +7586,10 @@
         <v>152</v>
       </c>
       <c r="B154" s="12" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D154" s="4" t="s">
         <v>16</v>
@@ -7610,13 +7611,13 @@
       </c>
       <c r="J154" s="8"/>
       <c r="K154" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L154" s="4">
         <v>6347</v>
       </c>
       <c r="M154" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="155" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7624,10 +7625,10 @@
         <v>153</v>
       </c>
       <c r="B155" s="12" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D155" s="4" t="s">
         <v>16</v>
@@ -7649,13 +7650,13 @@
       </c>
       <c r="J155" s="8"/>
       <c r="K155" s="17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L155" s="4">
         <v>6347</v>
       </c>
       <c r="M155" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="156" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7663,10 +7664,10 @@
         <v>154</v>
       </c>
       <c r="B156" s="11" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D156" s="4" t="s">
         <v>16</v>
@@ -7684,11 +7685,11 @@
         <v>93</v>
       </c>
       <c r="I156" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J156" s="8"/>
       <c r="K156" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L156" s="4">
         <v>6348</v>
@@ -7702,10 +7703,10 @@
         <v>155</v>
       </c>
       <c r="B157" s="11" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D157" s="4" t="s">
         <v>16</v>
@@ -7723,11 +7724,11 @@
         <v>93</v>
       </c>
       <c r="I157" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J157" s="8"/>
       <c r="K157" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L157" s="4">
         <v>6348</v>
@@ -7741,10 +7742,10 @@
         <v>156</v>
       </c>
       <c r="B158" s="12" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D158" s="4" t="s">
         <v>16</v>
@@ -7762,11 +7763,11 @@
         <v>93</v>
       </c>
       <c r="I158" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J158" s="8"/>
       <c r="K158" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L158" s="4">
         <v>6348</v>
@@ -7780,10 +7781,10 @@
         <v>157</v>
       </c>
       <c r="B159" s="12" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D159" s="4" t="s">
         <v>16</v>
@@ -7801,11 +7802,11 @@
         <v>93</v>
       </c>
       <c r="I159" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J159" s="8"/>
       <c r="K159" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L159" s="4">
         <v>6348</v>
@@ -7819,10 +7820,10 @@
         <v>158</v>
       </c>
       <c r="B160" s="11" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D160" s="4" t="s">
         <v>16</v>
@@ -7840,11 +7841,11 @@
         <v>93</v>
       </c>
       <c r="I160" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J160" s="8"/>
       <c r="K160" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L160" s="4">
         <v>6348</v>
@@ -7858,10 +7859,10 @@
         <v>159</v>
       </c>
       <c r="B161" s="12" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D161" s="4" t="s">
         <v>16</v>
@@ -7879,11 +7880,11 @@
         <v>713</v>
       </c>
       <c r="I161" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J161" s="8"/>
       <c r="K161" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L161" s="4">
         <v>6349</v>
@@ -7897,10 +7898,10 @@
         <v>160</v>
       </c>
       <c r="B162" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D162" s="4" t="s">
         <v>16</v>
@@ -7918,11 +7919,11 @@
         <v>713</v>
       </c>
       <c r="I162" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J162" s="8"/>
       <c r="K162" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L162" s="4">
         <v>6349</v>
@@ -7936,10 +7937,10 @@
         <v>161</v>
       </c>
       <c r="B163" s="12" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D163" s="4" t="s">
         <v>16</v>
@@ -7957,11 +7958,11 @@
         <v>6350</v>
       </c>
       <c r="I163" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J163" s="8"/>
       <c r="K163" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="L163" s="4">
         <v>6350</v>
@@ -7978,7 +7979,7 @@
         <v>45</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D164" s="4" t="s">
         <v>16</v>
@@ -7996,7 +7997,7 @@
         <v>26</v>
       </c>
       <c r="I164" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J164" s="8"/>
       <c r="K164" s="4" t="s">
@@ -8006,7 +8007,7 @@
         <v>6351</v>
       </c>
       <c r="M164" s="9" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="165" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8017,7 +8018,7 @@
         <v>45</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D165" s="4" t="s">
         <v>16</v>
@@ -8035,17 +8036,17 @@
         <v>141</v>
       </c>
       <c r="I165" s="9" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J165" s="8"/>
       <c r="K165" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L165" s="4">
         <v>6358</v>
       </c>
       <c r="M165" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="166" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8053,10 +8054,10 @@
         <v>164</v>
       </c>
       <c r="B166" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D166" s="4" t="s">
         <v>16</v>
@@ -8074,7 +8075,7 @@
         <v>1528</v>
       </c>
       <c r="I166" s="9" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J166" s="8"/>
       <c r="K166" s="4" t="s">
@@ -8084,7 +8085,7 @@
         <v>6359</v>
       </c>
       <c r="M166" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="167" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8092,10 +8093,10 @@
         <v>165</v>
       </c>
       <c r="B167" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D167" s="4" t="s">
         <v>16</v>
@@ -8113,7 +8114,7 @@
         <v>1528</v>
       </c>
       <c r="I167" s="9" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J167" s="8"/>
       <c r="K167" s="4" t="s">
@@ -8123,7 +8124,7 @@
         <v>6359</v>
       </c>
       <c r="M167" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="168" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8131,10 +8132,10 @@
         <v>166</v>
       </c>
       <c r="B168" s="11" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D168" s="4" t="s">
         <v>16</v>
@@ -8152,17 +8153,17 @@
         <v>142</v>
       </c>
       <c r="I168" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J168" s="8"/>
       <c r="K168" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L168" s="4">
         <v>6360</v>
       </c>
       <c r="M168" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="169" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8170,10 +8171,10 @@
         <v>167</v>
       </c>
       <c r="B169" s="11" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D169" s="4" t="s">
         <v>16</v>
@@ -8191,17 +8192,17 @@
         <v>142</v>
       </c>
       <c r="I169" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J169" s="8"/>
       <c r="K169" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L169" s="4">
         <v>6360</v>
       </c>
       <c r="M169" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="170" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8209,10 +8210,10 @@
         <v>168</v>
       </c>
       <c r="B170" s="11" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D170" s="4" t="s">
         <v>16</v>
@@ -8230,17 +8231,17 @@
         <v>143</v>
       </c>
       <c r="I170" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J170" s="8"/>
       <c r="K170" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="L170" s="4">
         <v>6361</v>
       </c>
       <c r="M170" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="171" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8248,10 +8249,10 @@
         <v>169</v>
       </c>
       <c r="B171" s="11" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D171" s="4" t="s">
         <v>16</v>
@@ -8269,17 +8270,17 @@
         <v>94</v>
       </c>
       <c r="I171" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J171" s="8"/>
       <c r="K171" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L171" s="4">
         <v>6362</v>
       </c>
       <c r="M171" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="172" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8288,7 +8289,7 @@
       </c>
       <c r="B172" s="12"/>
       <c r="C172" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D172" s="4" t="s">
         <v>16</v>
@@ -8306,17 +8307,17 @@
         <v>94</v>
       </c>
       <c r="I172" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J172" s="8"/>
       <c r="K172" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L172" s="4">
         <v>6362</v>
       </c>
       <c r="M172" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="173" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8324,10 +8325,10 @@
         <v>171</v>
       </c>
       <c r="B173" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D173" s="4" t="s">
         <v>16</v>
@@ -8345,17 +8346,17 @@
         <v>94</v>
       </c>
       <c r="I173" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J173" s="8"/>
       <c r="K173" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L173" s="4">
         <v>6362</v>
       </c>
       <c r="M173" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="174" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8363,10 +8364,10 @@
         <v>172</v>
       </c>
       <c r="B174" s="10" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D174" s="4" t="s">
         <v>16</v>
@@ -8384,17 +8385,17 @@
         <v>94</v>
       </c>
       <c r="I174" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J174" s="8"/>
       <c r="K174" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L174" s="4">
         <v>6362</v>
       </c>
       <c r="M174" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="175" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8402,10 +8403,10 @@
         <v>173</v>
       </c>
       <c r="B175" s="10" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D175" s="4" t="s">
         <v>16</v>
@@ -8423,17 +8424,17 @@
         <v>94</v>
       </c>
       <c r="I175" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J175" s="8"/>
       <c r="K175" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L175" s="4">
         <v>6362</v>
       </c>
       <c r="M175" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="176" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8441,10 +8442,10 @@
         <v>174</v>
       </c>
       <c r="B176" s="12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D176" s="4" t="s">
         <v>16</v>
@@ -8462,17 +8463,17 @@
         <v>14057</v>
       </c>
       <c r="I176" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J176" s="8"/>
       <c r="K176" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L176" s="4">
         <v>6363</v>
       </c>
       <c r="M176" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="177" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8480,10 +8481,10 @@
         <v>175</v>
       </c>
       <c r="B177" s="12" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D177" s="4" t="s">
         <v>16</v>
@@ -8501,17 +8502,17 @@
         <v>14057</v>
       </c>
       <c r="I177" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J177" s="8"/>
       <c r="K177" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L177" s="4">
         <v>6363</v>
       </c>
       <c r="M177" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="178" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8519,10 +8520,10 @@
         <v>176</v>
       </c>
       <c r="B178" s="12" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D178" s="4" t="s">
         <v>16</v>
@@ -8540,17 +8541,17 @@
         <v>14057</v>
       </c>
       <c r="I178" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J178" s="8"/>
       <c r="K178" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L178" s="4">
         <v>6363</v>
       </c>
       <c r="M178" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="179" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8561,7 +8562,7 @@
         <v>38</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D179" s="4" t="s">
         <v>16</v>
@@ -8579,7 +8580,7 @@
         <v>2464</v>
       </c>
       <c r="I179" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J179" s="8"/>
       <c r="K179" s="4" t="s">
@@ -8589,7 +8590,7 @@
         <v>6364</v>
       </c>
       <c r="M179" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="180" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8600,7 +8601,7 @@
         <v>49</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D180" s="4" t="s">
         <v>16</v>
@@ -8618,7 +8619,7 @@
         <v>2464</v>
       </c>
       <c r="I180" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J180" s="8"/>
       <c r="K180" s="4" t="s">
@@ -8628,7 +8629,7 @@
         <v>6364</v>
       </c>
       <c r="M180" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="181" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8636,10 +8637,10 @@
         <v>179</v>
       </c>
       <c r="B181" s="11" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D181" s="4" t="s">
         <v>16</v>
@@ -8657,7 +8658,7 @@
         <v>2464</v>
       </c>
       <c r="I181" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J181" s="8"/>
       <c r="K181" s="4" t="s">
@@ -8667,7 +8668,7 @@
         <v>6364</v>
       </c>
       <c r="M181" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="182" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8675,10 +8676,10 @@
         <v>180</v>
       </c>
       <c r="B182" s="11" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D182" s="4" t="s">
         <v>16</v>
@@ -8696,7 +8697,7 @@
         <v>2464</v>
       </c>
       <c r="I182" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J182" s="8"/>
       <c r="K182" s="4" t="s">
@@ -8706,7 +8707,7 @@
         <v>6364</v>
       </c>
       <c r="M182" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="183" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8717,7 +8718,7 @@
         <v>50</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D183" s="4" t="s">
         <v>16</v>
@@ -8735,7 +8736,7 @@
         <v>2464</v>
       </c>
       <c r="I183" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J183" s="8"/>
       <c r="K183" s="4" t="s">
@@ -8745,7 +8746,7 @@
         <v>6364</v>
       </c>
       <c r="M183" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="184" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8756,7 +8757,7 @@
         <v>47</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D184" s="4" t="s">
         <v>16</v>
@@ -8774,7 +8775,7 @@
         <v>2464</v>
       </c>
       <c r="I184" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J184" s="8"/>
       <c r="K184" s="4" t="s">
@@ -8784,7 +8785,7 @@
         <v>6364</v>
       </c>
       <c r="M184" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="185" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8792,10 +8793,10 @@
         <v>183</v>
       </c>
       <c r="B185" s="10" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D185" s="4" t="s">
         <v>16</v>
@@ -8813,7 +8814,7 @@
         <v>2464</v>
       </c>
       <c r="I185" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J185" s="8"/>
       <c r="K185" s="4" t="s">
@@ -8823,7 +8824,7 @@
         <v>6364</v>
       </c>
       <c r="M185" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="186" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8852,7 +8853,7 @@
         <v>2464</v>
       </c>
       <c r="I186" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J186" s="8"/>
       <c r="K186" s="4" t="s">
@@ -8862,7 +8863,7 @@
         <v>6364</v>
       </c>
       <c r="M186" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="187" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8870,10 +8871,10 @@
         <v>185</v>
       </c>
       <c r="B187" s="11" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D187" s="4" t="s">
         <v>16</v>
@@ -8891,7 +8892,7 @@
         <v>2464</v>
       </c>
       <c r="I187" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J187" s="8"/>
       <c r="K187" s="4" t="s">
@@ -8901,7 +8902,7 @@
         <v>6364</v>
       </c>
       <c r="M187" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="188" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8912,7 +8913,7 @@
         <v>42</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D188" s="4" t="s">
         <v>16</v>
@@ -8930,7 +8931,7 @@
         <v>2464</v>
       </c>
       <c r="I188" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J188" s="8"/>
       <c r="K188" s="4" t="s">
@@ -8940,7 +8941,7 @@
         <v>6364</v>
       </c>
       <c r="M188" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="189" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -8951,7 +8952,7 @@
         <v>43</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D189" s="4" t="s">
         <v>16</v>
@@ -8969,7 +8970,7 @@
         <v>2464</v>
       </c>
       <c r="I189" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J189" s="8"/>
       <c r="K189" s="4" t="s">
@@ -8979,7 +8980,7 @@
         <v>6364</v>
       </c>
       <c r="M189" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="190" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -9008,7 +9009,7 @@
         <v>2464</v>
       </c>
       <c r="I190" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J190" s="8"/>
       <c r="K190" s="4" t="s">
@@ -9018,7 +9019,7 @@
         <v>6364</v>
       </c>
       <c r="M190" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="191" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -9047,7 +9048,7 @@
         <v>2464</v>
       </c>
       <c r="I191" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J191" s="8"/>
       <c r="K191" s="4" t="s">
@@ -9057,7 +9058,7 @@
         <v>6365</v>
       </c>
       <c r="M191" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="192" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -9065,10 +9066,10 @@
         <v>190</v>
       </c>
       <c r="B192" s="10" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D192" s="4" t="s">
         <v>16</v>
@@ -9086,7 +9087,7 @@
         <v>2464</v>
       </c>
       <c r="I192" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J192" s="8"/>
       <c r="K192" s="4" t="s">
@@ -9096,7 +9097,7 @@
         <v>6365</v>
       </c>
       <c r="M192" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="193" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -9104,10 +9105,10 @@
         <v>191</v>
       </c>
       <c r="B193" s="10" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D193" s="4" t="s">
         <v>16</v>
@@ -9125,7 +9126,7 @@
         <v>2464</v>
       </c>
       <c r="I193" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J193" s="8"/>
       <c r="K193" s="4" t="s">
@@ -9135,7 +9136,7 @@
         <v>6365</v>
       </c>
       <c r="M193" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="194" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -9164,7 +9165,7 @@
         <v>2464</v>
       </c>
       <c r="I194" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J194" s="8"/>
       <c r="K194" s="4" t="s">
@@ -9174,7 +9175,7 @@
         <v>6365</v>
       </c>
       <c r="M194" s="9" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="195" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Update invoice and transaction Excel files with new revisions
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 5.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B8D029-F246-4018-BA47-4159023020F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51AD9B8-7B97-4B62-8E5C-D9102F3DA5F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="210" yWindow="3240" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="392">
   <si>
     <t>بورسعيد لصناعة المعادن</t>
   </si>
@@ -1210,6 +1210,9 @@
   </si>
   <si>
     <t>لوح 1.5 ﻣﻢ SST ﻣﺼﻨﻔﺮ ﻣﻐﻠﻒ 1.25 × 2 م</t>
+  </si>
+  <si>
+    <t>شركة الذهب للتيريد</t>
   </si>
 </sst>
 </file>
@@ -8052,7 +8055,7 @@
       </c>
       <c r="J163" s="8"/>
       <c r="K163" s="4" t="s">
-        <v>17</v>
+        <v>391</v>
       </c>
       <c r="L163" s="4">
         <v>6351</v>

</xml_diff>